<commit_message>
added poiji library to read the data from excel and make the excel reader class as generic
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/phoenix_test_data.xlsx
+++ b/src/test/resources/testData/phoenix_test_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tanagash\eclipse-workspace\PhoenixApiTestAutomation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97D7BC0-08B3-4CE6-973C-738C27BC3431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE41E2BE-9A2A-4FA8-A47B-FE90F69F96AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="3">
   <si>
     <t>username</t>
   </si>
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
@@ -390,38 +390,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added service utility for API
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/phoenix_test_data.xlsx
+++ b/src/test/resources/testData/phoenix_test_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tanagash\eclipse-workspace\PhoenixApiTestAutomation\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B81379-1393-4E92-8AE4-08BE3E9119E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760FCA73-6745-492B-9B43-004CC9426DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
   <si>
     <t>username</t>
   </si>
@@ -157,7 +157,37 @@
     <t>Ut illum autem</t>
   </si>
   <si>
-    <t>235601162186240</t>
+    <t>dhoni</t>
+  </si>
+  <si>
+    <t>mahendra</t>
+  </si>
+  <si>
+    <t>dhoni@hotmail.com</t>
+  </si>
+  <si>
+    <t>A-100</t>
+  </si>
+  <si>
+    <t>whisling Crossing</t>
+  </si>
+  <si>
+    <t>mankar Junction</t>
+  </si>
+  <si>
+    <t>BRT STOP</t>
+  </si>
+  <si>
+    <t>Kaspate wasti</t>
+  </si>
+  <si>
+    <t>india</t>
+  </si>
+  <si>
+    <t>battery iaaue</t>
+  </si>
+  <si>
+    <t>23561102186240</t>
   </si>
 </sst>
 </file>
@@ -551,7 +581,7 @@
     <col min="6" max="6" width="23.36328125" customWidth="1"/>
     <col min="7" max="7" width="25.81640625" customWidth="1"/>
     <col min="8" max="8" width="28.81640625" customWidth="1"/>
-    <col min="9" max="9" width="17.81640625" customWidth="1"/>
+    <col min="9" max="9" width="26.26953125" customWidth="1"/>
     <col min="10" max="10" width="21.90625" customWidth="1"/>
     <col min="11" max="11" width="30.90625" customWidth="1"/>
     <col min="12" max="12" width="33.08984375" customWidth="1"/>
@@ -679,10 +709,10 @@
       <c r="H2" s="1">
         <v>7747300082</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" t="s">
         <v>32</v>
       </c>
       <c r="K2" s="1" t="s">
@@ -713,13 +743,13 @@
         <v>40</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="W2" s="3" t="s">
         <v>41</v>
@@ -738,8 +768,87 @@
       </c>
     </row>
     <row r="3" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
+      <c r="A3" s="1">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="1">
+        <v>7747300123</v>
+      </c>
+      <c r="H3" s="1">
+        <v>7747300123</v>
+      </c>
+      <c r="I3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="P3" s="1">
+        <v>95790</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="W3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="X3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>12</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="4" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="T4" s="2"/>
@@ -748,6 +857,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="W2" r:id="rId1" display="www.advaya-sinha.in" xr:uid="{8954B304-508C-43C3-9F0F-61331272973F}"/>
+    <hyperlink ref="W3" r:id="rId2" display="www.advaya-sinha.in" xr:uid="{46E17A9F-C5DC-4672-BAAE-1E295D7A58BA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>